<commit_message>
fix(auth): eliminate /auth/callback hop — exchange PKCE code directly on reset-password page
The /auth/callback route.ts caused 404 in production because Next.js route
handlers are not always reliably hit by external redirects in Supabase's flow.

New approach: redirectTo points directly to /auth/reset-password. The page
detects ?code=, calls supabase.auth.exchangeCodeForSession(code) client-side,
then shows the form on success or an expired-link state on failure.

- Remove /auth/callback/route.ts entirely
- redirectTo: ${NEXT_PUBLIC_SITE_URL ?? origin}/auth/reset-password
- reset-password page: loading → exchange code → ready|invalid_link|success states
- Expired/invalid link shows clear Spanish message with back-to-login link

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/Reglas_Planificación.xlsx
+++ b/data/Reglas_Planificación.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/cami/Documents/Proyecto Producción ETP spa/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{78AF334C-56C3-9E4D-B75E-5181E5241805}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2C387CD8-79D3-994B-AB4F-9FFF56254346}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28800" yWindow="0" windowWidth="38400" windowHeight="21600" xr2:uid="{7437EE19-4B04-9348-BA7B-6D0EFE3DC538}"/>
+    <workbookView xWindow="0" yWindow="500" windowWidth="28800" windowHeight="16160" activeTab="1" xr2:uid="{7437EE19-4B04-9348-BA7B-6D0EFE3DC538}"/>
   </bookViews>
   <sheets>
     <sheet name="CÓDIGO PLAZO Y DEMORAS EN DÍAS" sheetId="7" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="45" uniqueCount="34">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="44" uniqueCount="33">
   <si>
     <t>Aljibe 10 m3</t>
   </si>
@@ -136,9 +136,6 @@
   </si>
   <si>
     <t>CAPACIDAD POR DÍA</t>
-  </si>
-  <si>
-    <t xml:space="preserve">arm1 , rem1, mont1 hacen combustible </t>
   </si>
 </sst>
 </file>
@@ -161,18 +158,12 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="2">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFFF00"/>
-        <bgColor indexed="64"/>
-      </patternFill>
     </fill>
   </fills>
   <borders count="4">
@@ -216,13 +207,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -538,7 +528,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{56C73070-36B1-BD45-84F0-686B9F2CAFBC}">
-  <dimension ref="A1:M23"/>
+  <dimension ref="A1:M18"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="17.1640625" customWidth="1"/>
@@ -554,37 +544,37 @@
       <c r="A1" t="s">
         <v>17</v>
       </c>
-      <c r="B1" s="6" t="s">
+      <c r="B1" t="s">
         <v>18</v>
       </c>
-      <c r="C1" s="6" t="s">
+      <c r="C1" t="s">
         <v>19</v>
       </c>
-      <c r="D1" s="6" t="s">
+      <c r="D1" t="s">
         <v>20</v>
       </c>
-      <c r="E1" s="6" t="s">
+      <c r="E1" t="s">
         <v>21</v>
       </c>
-      <c r="F1" s="6" t="s">
+      <c r="F1" t="s">
         <v>22</v>
       </c>
-      <c r="G1" s="6" t="s">
+      <c r="G1" t="s">
         <v>23</v>
       </c>
-      <c r="H1" s="6" t="s">
+      <c r="H1" t="s">
         <v>24</v>
       </c>
-      <c r="I1" s="6" t="s">
+      <c r="I1" t="s">
         <v>25</v>
       </c>
-      <c r="J1" s="6" t="s">
+      <c r="J1" t="s">
         <v>26</v>
       </c>
-      <c r="K1" s="6" t="s">
+      <c r="K1" t="s">
         <v>27</v>
       </c>
-      <c r="L1" s="6" t="s">
+      <c r="L1" t="s">
         <v>28</v>
       </c>
       <c r="M1" t="s">
@@ -595,37 +585,37 @@
       <c r="A2">
         <v>1</v>
       </c>
-      <c r="B2" s="6" t="s">
-        <v>0</v>
-      </c>
-      <c r="C2" s="6">
-        <v>1</v>
-      </c>
-      <c r="D2" s="6">
-        <v>1</v>
-      </c>
-      <c r="E2" s="6">
-        <v>1</v>
-      </c>
-      <c r="F2" s="6">
-        <v>1</v>
-      </c>
-      <c r="G2" s="6">
-        <v>2</v>
-      </c>
-      <c r="H2" s="6">
-        <v>2</v>
-      </c>
-      <c r="I2" s="6">
-        <v>1</v>
-      </c>
-      <c r="J2" s="6">
-        <v>1</v>
-      </c>
-      <c r="K2" s="6">
-        <v>1</v>
-      </c>
-      <c r="L2" s="6">
+      <c r="B2" t="s">
+        <v>0</v>
+      </c>
+      <c r="C2">
+        <v>1</v>
+      </c>
+      <c r="D2">
+        <v>1</v>
+      </c>
+      <c r="E2">
+        <v>1</v>
+      </c>
+      <c r="F2">
+        <v>1</v>
+      </c>
+      <c r="G2">
+        <v>2</v>
+      </c>
+      <c r="H2">
+        <v>2</v>
+      </c>
+      <c r="I2">
+        <v>1</v>
+      </c>
+      <c r="J2">
+        <v>1</v>
+      </c>
+      <c r="K2">
+        <v>1</v>
+      </c>
+      <c r="L2">
         <v>1</v>
       </c>
       <c r="M2">
@@ -636,37 +626,37 @@
       <c r="A3">
         <v>2</v>
       </c>
-      <c r="B3" s="6" t="s">
-        <v>1</v>
-      </c>
-      <c r="C3" s="6">
-        <v>1</v>
-      </c>
-      <c r="D3" s="6">
-        <v>1</v>
-      </c>
-      <c r="E3" s="6">
-        <v>1</v>
-      </c>
-      <c r="F3" s="6">
-        <v>2</v>
-      </c>
-      <c r="G3" s="6">
+      <c r="B3" t="s">
+        <v>1</v>
+      </c>
+      <c r="C3">
+        <v>1</v>
+      </c>
+      <c r="D3">
+        <v>1</v>
+      </c>
+      <c r="E3">
+        <v>1</v>
+      </c>
+      <c r="F3">
+        <v>2</v>
+      </c>
+      <c r="G3">
         <v>3</v>
       </c>
-      <c r="H3" s="6">
-        <v>2</v>
-      </c>
-      <c r="I3" s="6">
-        <v>2</v>
-      </c>
-      <c r="J3" s="6">
-        <v>2</v>
-      </c>
-      <c r="K3" s="6">
-        <v>1</v>
-      </c>
-      <c r="L3" s="6">
+      <c r="H3">
+        <v>2</v>
+      </c>
+      <c r="I3">
+        <v>2</v>
+      </c>
+      <c r="J3">
+        <v>2</v>
+      </c>
+      <c r="K3">
+        <v>1</v>
+      </c>
+      <c r="L3">
         <v>1</v>
       </c>
       <c r="M3">
@@ -677,37 +667,37 @@
       <c r="A4">
         <v>3</v>
       </c>
-      <c r="B4" s="6" t="s">
-        <v>2</v>
-      </c>
-      <c r="C4" s="6">
-        <v>1</v>
-      </c>
-      <c r="D4" s="6">
-        <v>1</v>
-      </c>
-      <c r="E4" s="6">
-        <v>0</v>
-      </c>
-      <c r="F4" s="6">
-        <v>0</v>
-      </c>
-      <c r="G4" s="6">
-        <v>2</v>
-      </c>
-      <c r="H4" s="6">
-        <v>2</v>
-      </c>
-      <c r="I4" s="6">
-        <v>1</v>
-      </c>
-      <c r="J4" s="6">
-        <v>1</v>
-      </c>
-      <c r="K4" s="6">
-        <v>1</v>
-      </c>
-      <c r="L4" s="6">
+      <c r="B4" t="s">
+        <v>2</v>
+      </c>
+      <c r="C4">
+        <v>1</v>
+      </c>
+      <c r="D4">
+        <v>1</v>
+      </c>
+      <c r="E4">
+        <v>0</v>
+      </c>
+      <c r="F4">
+        <v>0</v>
+      </c>
+      <c r="G4">
+        <v>2</v>
+      </c>
+      <c r="H4">
+        <v>2</v>
+      </c>
+      <c r="I4">
+        <v>1</v>
+      </c>
+      <c r="J4">
+        <v>1</v>
+      </c>
+      <c r="K4">
+        <v>1</v>
+      </c>
+      <c r="L4">
         <v>0</v>
       </c>
       <c r="M4">
@@ -718,37 +708,37 @@
       <c r="A5">
         <v>4</v>
       </c>
-      <c r="B5" s="6" t="s">
+      <c r="B5" t="s">
         <v>3</v>
       </c>
-      <c r="C5" s="6">
-        <v>1</v>
-      </c>
-      <c r="D5" s="6">
-        <v>1</v>
-      </c>
-      <c r="E5" s="6">
-        <v>1</v>
-      </c>
-      <c r="F5" s="6">
-        <v>1</v>
-      </c>
-      <c r="G5" s="6">
+      <c r="C5">
+        <v>1</v>
+      </c>
+      <c r="D5">
+        <v>1</v>
+      </c>
+      <c r="E5">
+        <v>1</v>
+      </c>
+      <c r="F5">
+        <v>1</v>
+      </c>
+      <c r="G5">
         <v>3</v>
       </c>
-      <c r="H5" s="6">
+      <c r="H5">
         <v>3</v>
       </c>
-      <c r="I5" s="6">
-        <v>1</v>
-      </c>
-      <c r="J5" s="6">
-        <v>1</v>
-      </c>
-      <c r="K5" s="6">
-        <v>1</v>
-      </c>
-      <c r="L5" s="6">
+      <c r="I5">
+        <v>1</v>
+      </c>
+      <c r="J5">
+        <v>1</v>
+      </c>
+      <c r="K5">
+        <v>1</v>
+      </c>
+      <c r="L5">
         <v>1</v>
       </c>
       <c r="M5">
@@ -759,37 +749,37 @@
       <c r="A6">
         <v>5</v>
       </c>
-      <c r="B6" s="6" t="s">
+      <c r="B6" t="s">
         <v>4</v>
       </c>
-      <c r="C6" s="6">
-        <v>1</v>
-      </c>
-      <c r="D6" s="6">
-        <v>1</v>
-      </c>
-      <c r="E6" s="6">
-        <v>1</v>
-      </c>
-      <c r="F6" s="6">
-        <v>1</v>
-      </c>
-      <c r="G6" s="6">
+      <c r="C6">
+        <v>1</v>
+      </c>
+      <c r="D6">
+        <v>1</v>
+      </c>
+      <c r="E6">
+        <v>1</v>
+      </c>
+      <c r="F6">
+        <v>1</v>
+      </c>
+      <c r="G6">
         <v>4</v>
       </c>
-      <c r="H6" s="6">
+      <c r="H6">
         <v>4</v>
       </c>
-      <c r="I6" s="6">
-        <v>2</v>
-      </c>
-      <c r="J6" s="6">
-        <v>2</v>
-      </c>
-      <c r="K6" s="6">
-        <v>1</v>
-      </c>
-      <c r="L6" s="6">
+      <c r="I6">
+        <v>2</v>
+      </c>
+      <c r="J6">
+        <v>2</v>
+      </c>
+      <c r="K6">
+        <v>1</v>
+      </c>
+      <c r="L6">
         <v>1</v>
       </c>
       <c r="M6">
@@ -800,37 +790,37 @@
       <c r="A7">
         <v>6</v>
       </c>
-      <c r="B7" s="6" t="s">
+      <c r="B7" t="s">
         <v>5</v>
       </c>
-      <c r="C7" s="6">
-        <v>1</v>
-      </c>
-      <c r="D7" s="6">
-        <v>1</v>
-      </c>
-      <c r="E7" s="6">
-        <v>1</v>
-      </c>
-      <c r="F7" s="6">
-        <v>1</v>
-      </c>
-      <c r="G7" s="6">
+      <c r="C7">
+        <v>1</v>
+      </c>
+      <c r="D7">
+        <v>1</v>
+      </c>
+      <c r="E7">
+        <v>1</v>
+      </c>
+      <c r="F7">
+        <v>1</v>
+      </c>
+      <c r="G7">
         <v>3</v>
       </c>
-      <c r="H7" s="6">
-        <v>0</v>
-      </c>
-      <c r="I7" s="6">
-        <v>2</v>
-      </c>
-      <c r="J7" s="6">
-        <v>1</v>
-      </c>
-      <c r="K7" s="6">
-        <v>1</v>
-      </c>
-      <c r="L7" s="6">
+      <c r="H7">
+        <v>0</v>
+      </c>
+      <c r="I7">
+        <v>2</v>
+      </c>
+      <c r="J7">
+        <v>1</v>
+      </c>
+      <c r="K7">
+        <v>1</v>
+      </c>
+      <c r="L7">
         <v>1</v>
       </c>
       <c r="M7">
@@ -841,37 +831,37 @@
       <c r="A8">
         <v>7</v>
       </c>
-      <c r="B8" s="6" t="s">
+      <c r="B8" t="s">
         <v>6</v>
       </c>
-      <c r="C8" s="6">
-        <v>2</v>
-      </c>
-      <c r="D8" s="6">
-        <v>2</v>
-      </c>
-      <c r="E8" s="6">
-        <v>2</v>
-      </c>
-      <c r="F8" s="6">
+      <c r="C8">
+        <v>2</v>
+      </c>
+      <c r="D8">
+        <v>2</v>
+      </c>
+      <c r="E8">
+        <v>2</v>
+      </c>
+      <c r="F8">
         <v>3</v>
       </c>
-      <c r="G8" s="6">
+      <c r="G8">
         <v>5</v>
       </c>
-      <c r="H8" s="6">
-        <v>1</v>
-      </c>
-      <c r="I8" s="6">
-        <v>2</v>
-      </c>
-      <c r="J8" s="6">
-        <v>2</v>
-      </c>
-      <c r="K8" s="6">
-        <v>1</v>
-      </c>
-      <c r="L8" s="6">
+      <c r="H8">
+        <v>1</v>
+      </c>
+      <c r="I8">
+        <v>2</v>
+      </c>
+      <c r="J8">
+        <v>2</v>
+      </c>
+      <c r="K8">
+        <v>1</v>
+      </c>
+      <c r="L8">
         <v>2</v>
       </c>
       <c r="M8">
@@ -882,37 +872,37 @@
       <c r="A9">
         <v>8</v>
       </c>
-      <c r="B9" s="6" t="s">
+      <c r="B9" t="s">
         <v>7</v>
       </c>
-      <c r="C9" s="6">
-        <v>1</v>
-      </c>
-      <c r="D9" s="6">
-        <v>1</v>
-      </c>
-      <c r="E9" s="6">
-        <v>1</v>
-      </c>
-      <c r="F9" s="6">
-        <v>2</v>
-      </c>
-      <c r="G9" s="6">
-        <v>2</v>
-      </c>
-      <c r="H9" s="6">
-        <v>1</v>
-      </c>
-      <c r="I9" s="6">
-        <v>1</v>
-      </c>
-      <c r="J9" s="6">
-        <v>1</v>
-      </c>
-      <c r="K9" s="6">
-        <v>1</v>
-      </c>
-      <c r="L9" s="6">
+      <c r="C9">
+        <v>1</v>
+      </c>
+      <c r="D9">
+        <v>1</v>
+      </c>
+      <c r="E9">
+        <v>1</v>
+      </c>
+      <c r="F9">
+        <v>2</v>
+      </c>
+      <c r="G9">
+        <v>2</v>
+      </c>
+      <c r="H9">
+        <v>1</v>
+      </c>
+      <c r="I9">
+        <v>1</v>
+      </c>
+      <c r="J9">
+        <v>1</v>
+      </c>
+      <c r="K9">
+        <v>1</v>
+      </c>
+      <c r="L9">
         <v>1</v>
       </c>
       <c r="M9">
@@ -923,37 +913,37 @@
       <c r="A10">
         <v>9</v>
       </c>
-      <c r="B10" s="6" t="s">
+      <c r="B10" t="s">
         <v>8</v>
       </c>
-      <c r="C10" s="6">
-        <v>2</v>
-      </c>
-      <c r="D10" s="6">
-        <v>1</v>
-      </c>
-      <c r="E10" s="6">
-        <v>1</v>
-      </c>
-      <c r="F10" s="6">
+      <c r="C10">
+        <v>2</v>
+      </c>
+      <c r="D10">
+        <v>1</v>
+      </c>
+      <c r="E10">
+        <v>1</v>
+      </c>
+      <c r="F10">
         <v>4</v>
       </c>
-      <c r="G10" s="6">
+      <c r="G10">
         <v>5</v>
       </c>
-      <c r="H10" s="6">
+      <c r="H10">
         <v>6</v>
       </c>
-      <c r="I10" s="6">
-        <v>2</v>
-      </c>
-      <c r="J10" s="6">
+      <c r="I10">
+        <v>2</v>
+      </c>
+      <c r="J10">
         <v>5</v>
       </c>
-      <c r="K10" s="6">
-        <v>1</v>
-      </c>
-      <c r="L10" s="6">
+      <c r="K10">
+        <v>1</v>
+      </c>
+      <c r="L10">
         <v>2</v>
       </c>
       <c r="M10">
@@ -964,37 +954,37 @@
       <c r="A11">
         <v>10</v>
       </c>
-      <c r="B11" s="6" t="s">
+      <c r="B11" t="s">
         <v>9</v>
       </c>
-      <c r="C11" s="6">
-        <v>2</v>
-      </c>
-      <c r="D11" s="6">
-        <v>1</v>
-      </c>
-      <c r="E11" s="6">
-        <v>1</v>
-      </c>
-      <c r="F11" s="6">
+      <c r="C11">
+        <v>2</v>
+      </c>
+      <c r="D11">
+        <v>1</v>
+      </c>
+      <c r="E11">
+        <v>1</v>
+      </c>
+      <c r="F11">
         <v>3</v>
       </c>
-      <c r="G11" s="6">
+      <c r="G11">
         <v>5</v>
       </c>
-      <c r="H11" s="6">
+      <c r="H11">
         <v>4</v>
       </c>
-      <c r="I11" s="6">
-        <v>2</v>
-      </c>
-      <c r="J11" s="6">
+      <c r="I11">
+        <v>2</v>
+      </c>
+      <c r="J11">
         <v>5</v>
       </c>
-      <c r="K11" s="6">
-        <v>1</v>
-      </c>
-      <c r="L11" s="6">
+      <c r="K11">
+        <v>1</v>
+      </c>
+      <c r="L11">
         <v>2</v>
       </c>
       <c r="M11">
@@ -1005,37 +995,37 @@
       <c r="A12">
         <v>11</v>
       </c>
-      <c r="B12" s="6" t="s">
+      <c r="B12" t="s">
         <v>10</v>
       </c>
-      <c r="C12" s="6">
-        <v>1</v>
-      </c>
-      <c r="D12" s="6">
-        <v>1</v>
-      </c>
-      <c r="E12" s="6">
-        <v>1</v>
-      </c>
-      <c r="F12" s="6">
-        <v>0</v>
-      </c>
-      <c r="G12" s="6">
-        <v>2</v>
-      </c>
-      <c r="H12" s="6">
-        <v>2</v>
-      </c>
-      <c r="I12" s="6">
-        <v>1</v>
-      </c>
-      <c r="J12" s="6">
-        <v>1</v>
-      </c>
-      <c r="K12" s="6">
-        <v>1</v>
-      </c>
-      <c r="L12" s="6">
+      <c r="C12">
+        <v>1</v>
+      </c>
+      <c r="D12">
+        <v>1</v>
+      </c>
+      <c r="E12">
+        <v>1</v>
+      </c>
+      <c r="F12">
+        <v>0</v>
+      </c>
+      <c r="G12">
+        <v>2</v>
+      </c>
+      <c r="H12">
+        <v>2</v>
+      </c>
+      <c r="I12">
+        <v>1</v>
+      </c>
+      <c r="J12">
+        <v>1</v>
+      </c>
+      <c r="K12">
+        <v>1</v>
+      </c>
+      <c r="L12">
         <v>0</v>
       </c>
       <c r="M12">
@@ -1046,37 +1036,37 @@
       <c r="A13">
         <v>12</v>
       </c>
-      <c r="B13" s="6" t="s">
+      <c r="B13" t="s">
         <v>11</v>
       </c>
-      <c r="C13" s="6">
-        <v>2</v>
-      </c>
-      <c r="D13" s="6">
-        <v>1</v>
-      </c>
-      <c r="E13" s="6">
-        <v>1</v>
-      </c>
-      <c r="F13" s="6">
+      <c r="C13">
+        <v>2</v>
+      </c>
+      <c r="D13">
+        <v>1</v>
+      </c>
+      <c r="E13">
+        <v>1</v>
+      </c>
+      <c r="F13">
         <v>4</v>
       </c>
-      <c r="G13" s="6">
+      <c r="G13">
         <v>6</v>
       </c>
-      <c r="H13" s="6">
+      <c r="H13">
         <v>25</v>
       </c>
-      <c r="I13" s="6">
+      <c r="I13">
         <v>3</v>
       </c>
-      <c r="J13" s="6">
+      <c r="J13">
         <v>5</v>
       </c>
-      <c r="K13" s="6">
-        <v>1</v>
-      </c>
-      <c r="L13" s="6">
+      <c r="K13">
+        <v>1</v>
+      </c>
+      <c r="L13">
         <v>2</v>
       </c>
       <c r="M13">
@@ -1087,37 +1077,37 @@
       <c r="A14">
         <v>13</v>
       </c>
-      <c r="B14" s="6" t="s">
+      <c r="B14" t="s">
         <v>12</v>
       </c>
-      <c r="C14" s="6">
-        <v>1</v>
-      </c>
-      <c r="D14" s="6">
-        <v>1</v>
-      </c>
-      <c r="E14" s="6">
-        <v>1</v>
-      </c>
-      <c r="F14" s="6">
-        <v>1</v>
-      </c>
-      <c r="G14" s="6">
+      <c r="C14">
+        <v>1</v>
+      </c>
+      <c r="D14">
+        <v>1</v>
+      </c>
+      <c r="E14">
+        <v>1</v>
+      </c>
+      <c r="F14">
+        <v>1</v>
+      </c>
+      <c r="G14">
         <v>3</v>
       </c>
-      <c r="H14" s="6">
+      <c r="H14">
         <v>8</v>
       </c>
-      <c r="I14" s="6">
-        <v>2</v>
-      </c>
-      <c r="J14" s="6">
+      <c r="I14">
+        <v>2</v>
+      </c>
+      <c r="J14">
         <v>3</v>
       </c>
-      <c r="K14" s="6">
-        <v>1</v>
-      </c>
-      <c r="L14" s="6">
+      <c r="K14">
+        <v>1</v>
+      </c>
+      <c r="L14">
         <v>1</v>
       </c>
       <c r="M14">
@@ -1128,37 +1118,37 @@
       <c r="A15">
         <v>14</v>
       </c>
-      <c r="B15" s="6" t="s">
+      <c r="B15" t="s">
         <v>13</v>
       </c>
-      <c r="C15" s="6">
-        <v>2</v>
-      </c>
-      <c r="D15" s="6">
-        <v>1</v>
-      </c>
-      <c r="E15" s="6">
-        <v>1</v>
-      </c>
-      <c r="F15" s="6">
-        <v>2</v>
-      </c>
-      <c r="G15" s="6">
+      <c r="C15">
+        <v>2</v>
+      </c>
+      <c r="D15">
+        <v>1</v>
+      </c>
+      <c r="E15">
+        <v>1</v>
+      </c>
+      <c r="F15">
+        <v>2</v>
+      </c>
+      <c r="G15">
         <v>3</v>
       </c>
-      <c r="H15" s="6">
+      <c r="H15">
         <v>12</v>
       </c>
-      <c r="I15" s="6">
-        <v>2</v>
-      </c>
-      <c r="J15" s="6">
+      <c r="I15">
+        <v>2</v>
+      </c>
+      <c r="J15">
         <v>4</v>
       </c>
-      <c r="K15" s="6">
-        <v>1</v>
-      </c>
-      <c r="L15" s="6">
+      <c r="K15">
+        <v>1</v>
+      </c>
+      <c r="L15">
         <v>1</v>
       </c>
       <c r="M15">
@@ -1286,11 +1276,6 @@
       </c>
       <c r="M18">
         <v>0</v>
-      </c>
-    </row>
-    <row r="23" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="C23" t="s">
-        <v>33</v>
       </c>
     </row>
   </sheetData>
@@ -1369,7 +1354,7 @@
       <c r="B6">
         <v>5</v>
       </c>
-      <c r="C6">
+      <c r="C6" s="5">
         <v>2</v>
       </c>
     </row>

</xml_diff>